<commit_message>
feat: remove R2 storage and branding settings, set default static logo.png
</commit_message>
<xml_diff>
--- a/HRM_Database_Normalized.xlsx
+++ b/HRM_Database_Normalized.xlsx
@@ -654,10 +654,69 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+  <dimension ref="A1:I2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>log_id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>timestamp</v>
+      </c>
+      <c r="C1" t="str">
+        <v>user_id</v>
+      </c>
+      <c r="D1" t="str">
+        <v>user_name</v>
+      </c>
+      <c r="E1" t="str">
+        <v>user_role</v>
+      </c>
+      <c r="F1" t="str">
+        <v>action_type</v>
+      </c>
+      <c r="G1" t="str">
+        <v>module</v>
+      </c>
+      <c r="H1" t="str">
+        <v>description</v>
+      </c>
+      <c r="I1" t="str">
+        <v>ip_address</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>LOG-1788744799013-527</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-09-07T01:33:19.013Z</v>
+      </c>
+      <c r="C2" t="str">
+        <v>TH-1948</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Huỳnh Thanh Long</v>
+      </c>
+      <c r="E2" t="str">
+        <v>ADMIN</v>
+      </c>
+      <c r="F2" t="str">
+        <v>LOGIN</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Bảo mật</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Đăng nhập thành công vào hệ thống (Huỳnh Thanh Long - Quyền: ADMIN)</v>
+      </c>
+      <c r="I2" t="str">
+        <v>::1</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>